<commit_message>
fix(units): petrochemical electricity in MWh, shipping fuels in t
- petrochemical: Electricity modelled in MWh (intensity kWh/t ÷1000, price ×1000
  to $/MWh, grid emission native tCO2/MWh, NCC-Electricity native MWh/t); other
  energy GJ, H2/product in t
- shipping: fuel mass unit relabelled MT → t
- steel energy stays GJ (electricity shares a fuel blend group with H2; a group
  must be single-unit for the energy shares to be meaningful) — feedstocks in t
- both regenerated; objective unchanged (unit conversion is consistent)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/pathwise/public/examples/petrochemical.xlsx
+++ b/frontend/pathwise/public/examples/petrochemical.xlsx
@@ -1239,7 +1239,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kWh</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
         <v>16</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I2" t="n">
         <v>6730.751129518071</v>
@@ -1424,7 +1424,7 @@
         <v>16</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I3" t="n">
         <v>5878.319343550674</v>
@@ -1453,7 +1453,7 @@
         <v>16</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I4" t="n">
         <v>5015.38230126388</v>
@@ -1482,7 +1482,7 @@
         <v>16</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I5" t="n">
         <v>4162.95051529648</v>
@@ -1511,7 +1511,7 @@
         <v>16</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I6" t="n">
         <v>3310.517806520199</v>
@@ -1540,7 +1540,7 @@
         <v>16</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I7" t="n">
         <v>2626.159970765414</v>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.000436</v>
+        <v>0.436</v>
       </c>
     </row>
     <row r="4">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>46.16084915216484</v>
+        <v>0.04616084915216485</v>
       </c>
       <c r="E2" t="inlineStr"/>
     </row>
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>54.85338441425868</v>
+        <v>0.05485338441425869</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
@@ -2148,7 +2148,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5000</v>
+        <v>5</v>
       </c>
       <c r="E15" t="inlineStr"/>
     </row>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1.086461625741636</v>
+        <v>0.001086461625741636</v>
       </c>
       <c r="E17" t="inlineStr"/>
     </row>

</xml_diff>